<commit_message>
Day 3: Project 1 requirements
</commit_message>
<xml_diff>
--- a/niasap-data.xlsx
+++ b/niasap-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/metodiuswaruwu/Documents/Project AI/AI-Portofolio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E37969DF-138F-B44A-9316-15A70041569A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4251BB3-854A-4E40-BFF7-95AEAC76B197}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16100" yWindow="660" windowWidth="12620" windowHeight="17160" activeTab="3" xr2:uid="{9BF11571-3D57-C340-BE5B-8CD2BEA4A557}"/>
+    <workbookView xWindow="10940" yWindow="660" windowWidth="17780" windowHeight="17160" activeTab="3" xr2:uid="{9BF11571-3D57-C340-BE5B-8CD2BEA4A557}"/>
   </bookViews>
   <sheets>
     <sheet name="Sales" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Fix Cost" sheetId="3" r:id="rId3"/>
     <sheet name="Category" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="48">
   <si>
     <t>Tanggal</t>
   </si>
@@ -83,9 +83,6 @@
     <t>Bahan Baku</t>
   </si>
   <si>
-    <t>November</t>
-  </si>
-  <si>
     <t>Sewa</t>
   </si>
   <si>
@@ -146,9 +143,6 @@
     <t>Gas 5 kg</t>
   </si>
   <si>
-    <t>Belanja kebutuhan Minggu 1 November</t>
-  </si>
-  <si>
     <t>Bumbu Dapur paket</t>
   </si>
   <si>
@@ -182,9 +176,6 @@
     <t>Weekend hari keluarga</t>
   </si>
   <si>
-    <t>y</t>
-  </si>
-  <si>
     <t>Mahasiswa dan paket murah banyak laku</t>
   </si>
   <si>
@@ -192,6 +183,9 @@
   </si>
   <si>
     <t>Mendung dan hujan</t>
+  </si>
+  <si>
+    <t>Date</t>
   </si>
 </sst>
 </file>
@@ -572,7 +566,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0BD2659-175E-4540-A502-3A88DE202416}">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.5" bestFit="1" customWidth="1"/>
@@ -625,7 +619,7 @@
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -648,7 +642,7 @@
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -665,13 +659,13 @@
         <v>600000</v>
       </c>
       <c r="E4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F4">
         <v>20000</v>
       </c>
       <c r="G4" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -688,13 +682,13 @@
         <v>250000</v>
       </c>
       <c r="E5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F5">
         <v>200000</v>
       </c>
       <c r="G5" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -711,13 +705,13 @@
         <v>250000</v>
       </c>
       <c r="E6" t="s">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="F6">
         <v>0</v>
       </c>
       <c r="G6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -740,7 +734,7 @@
         <v>0</v>
       </c>
       <c r="G7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -763,49 +757,7 @@
         <v>0</v>
       </c>
       <c r="G8" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B15">
-        <f>SUM(B2:D2)</f>
-        <v>2000000</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B16">
-        <f t="shared" ref="B16:B21" si="0">SUM(B3:D3)</f>
-        <v>1950000</v>
-      </c>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B17">
-        <f t="shared" si="0"/>
-        <v>1920000</v>
-      </c>
-    </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B18">
-        <f t="shared" si="0"/>
-        <v>1800000</v>
-      </c>
-    </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B19">
-        <f t="shared" si="0"/>
-        <v>1550000</v>
-      </c>
-    </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B20">
-        <f t="shared" si="0"/>
-        <v>2000000</v>
-      </c>
-    </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B21">
-        <f t="shared" si="0"/>
-        <v>2000000</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -815,7 +767,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{136813CC-4999-A642-BE3F-F98151738BFA}">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.5" bestFit="1" customWidth="1"/>
@@ -825,24 +777,36 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>34</v>
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>0</v>
+      <c r="A2" s="1">
+        <v>46326</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" t="s">
-        <v>10</v>
+        <v>39</v>
+      </c>
+      <c r="D2">
+        <v>5000000</v>
       </c>
       <c r="E2" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -853,13 +817,13 @@
         <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D3">
-        <v>5000000</v>
+        <v>450000</v>
       </c>
       <c r="E3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -867,16 +831,16 @@
         <v>46326</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
         <v>27</v>
       </c>
       <c r="D4">
-        <v>450000</v>
+        <v>100000</v>
       </c>
       <c r="E4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -884,16 +848,16 @@
         <v>46326</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D5">
-        <v>100000</v>
+        <v>25000</v>
       </c>
       <c r="E5" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -901,16 +865,16 @@
         <v>46326</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D6">
-        <v>25000</v>
+        <v>80000</v>
       </c>
       <c r="E6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -921,13 +885,13 @@
         <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D7">
-        <v>80000</v>
+        <v>20000</v>
       </c>
       <c r="E7" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -935,16 +899,16 @@
         <v>46326</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="C8" t="s">
         <v>33</v>
       </c>
       <c r="D8">
-        <v>20000</v>
+        <v>250000</v>
       </c>
       <c r="E8" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -952,16 +916,16 @@
         <v>46326</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="C9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D9">
-        <v>250000</v>
+        <v>50000</v>
       </c>
       <c r="E9" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
@@ -972,13 +936,13 @@
         <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D10">
         <v>50000</v>
       </c>
       <c r="E10" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
@@ -986,33 +950,33 @@
         <v>46326</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="C11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D11">
-        <v>50000</v>
+        <v>100000</v>
       </c>
       <c r="E11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="B12" t="s">
         <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D12">
-        <v>100000</v>
+        <v>250000</v>
       </c>
       <c r="E12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
@@ -1020,33 +984,16 @@
         <v>46327</v>
       </c>
       <c r="B13" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="C13" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D13">
-        <v>250000</v>
+        <v>100000</v>
       </c>
       <c r="E13" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="1">
-        <v>46327</v>
-      </c>
-      <c r="B14" t="s">
-        <v>29</v>
-      </c>
-      <c r="C14" t="s">
-        <v>32</v>
-      </c>
-      <c r="D14">
-        <v>100000</v>
-      </c>
-      <c r="E14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -1056,112 +1003,143 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9A2E5AF-02BC-D441-AA8F-C555626022DF}">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A2:C13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <v>46328</v>
+      </c>
+      <c r="B3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3">
+      <c r="C3">
         <f>15000000/12</f>
         <v>1250000</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
+        <v>46328</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4">
+        <v>203000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
+        <v>46328</v>
+      </c>
+      <c r="B5" t="s">
         <v>15</v>
       </c>
-      <c r="B4">
-        <v>203000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="C5">
+        <v>319150</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
+        <v>46328</v>
+      </c>
+      <c r="B6" t="s">
         <v>16</v>
       </c>
-      <c r="B5">
-        <v>319150</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="C6">
+        <v>259475</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
+        <v>46332</v>
+      </c>
+      <c r="B7" t="s">
         <v>17</v>
       </c>
-      <c r="B6">
-        <v>259475</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7">
+      <c r="C7">
         <v>1600000</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
+        <v>46332</v>
+      </c>
+      <c r="B8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8">
+        <v>102500</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
+        <v>46332</v>
+      </c>
+      <c r="B9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
+        <v>46332</v>
+      </c>
+      <c r="B10" t="s">
         <v>21</v>
       </c>
-      <c r="B8">
-        <v>102500</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9">
-        <v>100000</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+      <c r="C10">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
+        <v>46336</v>
+      </c>
+      <c r="B11" t="s">
         <v>22</v>
       </c>
-      <c r="B10">
-        <v>25000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="C11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="1">
+        <v>46337</v>
+      </c>
+      <c r="B12" t="s">
         <v>23</v>
       </c>
-      <c r="B11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+      <c r="C12">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="1">
+        <v>46338</v>
+      </c>
+      <c r="B13" t="s">
         <v>24</v>
       </c>
-      <c r="B12">
-        <v>250000</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>25</v>
-      </c>
-      <c r="B13">
+      <c r="C13">
         <v>250000</v>
       </c>
     </row>
@@ -1172,7 +1150,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F160D3D0-3C84-5A42-AA19-77A6DA48B828}">
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -1183,6 +1161,11 @@
         <v>8</v>
       </c>
     </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>29</v>
@@ -1190,12 +1173,12 @@
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
-        <v>12</v>
+      <c r="A5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
@@ -1220,17 +1203,17 @@
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
@@ -1246,11 +1229,6 @@
     <row r="15" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>24</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Day 5: dashboard skeleton with KPIs and payment split
</commit_message>
<xml_diff>
--- a/niasap-data.xlsx
+++ b/niasap-data.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/metodiuswaruwu/Documents/Project AI/AI-Portofolio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4251BB3-854A-4E40-BFF7-95AEAC76B197}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70C48403-C433-BE4E-8179-A35AE72EAFC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10940" yWindow="660" windowWidth="17780" windowHeight="17160" activeTab="3" xr2:uid="{9BF11571-3D57-C340-BE5B-8CD2BEA4A557}"/>
+    <workbookView xWindow="16500" yWindow="660" windowWidth="12220" windowHeight="17160" activeTab="4" xr2:uid="{9BF11571-3D57-C340-BE5B-8CD2BEA4A557}"/>
   </bookViews>
   <sheets>
     <sheet name="Sales" sheetId="1" r:id="rId1"/>
     <sheet name="Expense" sheetId="2" r:id="rId2"/>
     <sheet name="Fix Cost" sheetId="3" r:id="rId3"/>
     <sheet name="Category" sheetId="4" r:id="rId4"/>
+    <sheet name="Dashboard" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,8 +42,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="59">
   <si>
     <t>Tanggal</t>
   </si>
@@ -186,13 +209,49 @@
   </si>
   <si>
     <t>Date</t>
+  </si>
+  <si>
+    <t>KPI</t>
+  </si>
+  <si>
+    <t>Total Pendapatan</t>
+  </si>
+  <si>
+    <t>Total Pengeluaran</t>
+  </si>
+  <si>
+    <t>Laba / Rugi</t>
+  </si>
+  <si>
+    <t>Margin %</t>
+  </si>
+  <si>
+    <t>Total Waste</t>
+  </si>
+  <si>
+    <t>Payment Method Split</t>
+  </si>
+  <si>
+    <t>QRIS</t>
+  </si>
+  <si>
+    <t>Grafik Pendapatan Harian</t>
+  </si>
+  <si>
+    <t>Breakdown Pengeluaran per Kategori</t>
+  </si>
+  <si>
+    <t>Tren Waste</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -205,6 +264,20 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -225,18 +298,54 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1234,4 +1343,132 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8990D63A-A126-C24A-9B4A-765D86C2F454}">
+  <dimension ref="A1:F30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" s="5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B3" s="4">
+        <f>SUM(Sales!B2:D8)</f>
+        <v>13220000</v>
+      </c>
+      <c r="C3" s="4" cm="1">
+        <f t="array" ref="C3">SUM(Expense!D2:D13+'Fix Cost'!C3:C14)</f>
+        <v>10834125</v>
+      </c>
+      <c r="D3" s="4">
+        <f>B3-C3</f>
+        <v>2385875</v>
+      </c>
+      <c r="E3" s="3">
+        <f>IF(B3=0,0,D3/B3)</f>
+        <v>0.18047465960665657</v>
+      </c>
+      <c r="F3" s="4">
+        <f>SUM(Sales!F2:F8)</f>
+        <v>220000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" s="5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B7" s="4">
+        <f>SUM(Sales!B2:B8)</f>
+        <v>5950000</v>
+      </c>
+      <c r="C7" s="4">
+        <f>SUM(Sales!C2:C8)</f>
+        <v>4620000</v>
+      </c>
+      <c r="D7" s="4">
+        <f>SUM(Sales!D2:D8)</f>
+        <v>2650000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B8" s="3">
+        <f>SUM(Sales!B2:B8)/B3</f>
+        <v>0.45007564296520425</v>
+      </c>
+      <c r="C8" s="3">
+        <f>SUM(Sales!C2:C8)/B3</f>
+        <v>0.34947049924357032</v>
+      </c>
+      <c r="D8" s="3">
+        <f>SUM(Sales!D2:D8)/B3</f>
+        <v>0.2004538577912254</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="D3">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Day 6: dashboard charts
</commit_message>
<xml_diff>
--- a/niasap-data.xlsx
+++ b/niasap-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/metodiuswaruwu/Documents/Project AI/AI-Portofolio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70C48403-C433-BE4E-8179-A35AE72EAFC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F445EF8E-99E9-1745-B6F6-C18C020F2036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16500" yWindow="660" windowWidth="12220" windowHeight="17160" activeTab="4" xr2:uid="{9BF11571-3D57-C340-BE5B-8CD2BEA4A557}"/>
+    <workbookView xWindow="16680" yWindow="660" windowWidth="12040" windowHeight="17160" activeTab="4" xr2:uid="{9BF11571-3D57-C340-BE5B-8CD2BEA4A557}"/>
   </bookViews>
   <sheets>
     <sheet name="Sales" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,10 @@
     <sheet name="Category" sheetId="4" r:id="rId4"/>
     <sheet name="Dashboard" sheetId="5" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v2.0" hidden="1">Sales!$A$2:$A$8</definedName>
+    <definedName name="_xlchart.v2.1" hidden="1">Sales!$F$2:$F$8</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -65,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="59">
   <si>
     <t>Tanggal</t>
   </si>
@@ -356,6 +360,2878 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Sales</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:areaChart>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sales!$A$2:$A$8</c:f>
+              <c:numCache>
+                <c:formatCode>m/d/yy</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>46328</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46329</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46330</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>46331</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>46332</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>46333</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>46334</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sales!$B$2:$B$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>1200000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>500000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1200000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>750000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>600000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>500000</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1200000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-0E6A-5049-84F3-89B292C7DAC0}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sales!$A$2:$A$8</c:f>
+              <c:numCache>
+                <c:formatCode>m/d/yy</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>46328</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46329</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46330</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>46331</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>46332</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>46333</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>46334</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sales!$C$2:$C$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>250000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1200000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>120000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>800000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>700000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1300000</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>250000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-0E6A-5049-84F3-89B292C7DAC0}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent3"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sales!$A$2:$A$8</c:f>
+              <c:numCache>
+                <c:formatCode>m/d/yy</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>46328</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46329</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46330</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>46331</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>46332</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>46333</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>46334</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sales!$D$2:$D$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>550000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>250000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>600000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>250000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>250000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>200000</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>550000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-0E6A-5049-84F3-89B292C7DAC0}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1312384192"/>
+        <c:axId val="1391876672"/>
+      </c:areaChart>
+      <c:dateAx>
+        <c:axId val="1312384192"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="m/d/yy" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1391876672"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblOffset val="100"/>
+        <c:baseTimeUnit val="days"/>
+      </c:dateAx>
+      <c:valAx>
+        <c:axId val="1391876672"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1312384192"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="zero"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Expanse</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>Dashboard!$H$21:$H$23</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Bahan Minum</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Bahan Masak</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Bahan Baku</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$I$21:$I$23</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>355000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>70000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6050000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-1FA6-4E46-A285-864C8CC02D1E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Waste</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sales!$A$2:$A$8</c:f>
+              <c:numCache>
+                <c:formatCode>m/d/yy</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>46328</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46329</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46330</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>46331</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>46332</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>46333</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>46334</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sales!$F$2:$F$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>20000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>200000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-DBF9-944A-BDAC-F100023B0792}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="1389997888"/>
+        <c:axId val="1389986240"/>
+      </c:lineChart>
+      <c:dateAx>
+        <c:axId val="1389997888"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="m/d/yy" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1389986240"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblOffset val="100"/>
+        <c:baseTimeUnit val="days"/>
+      </c:dateAx>
+      <c:valAx>
+        <c:axId val="1389986240"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1389997888"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="276">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>812800</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F1800911-18C7-DF4D-A07E-2FC8A27B281B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>63500</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>203200</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C566CDED-D31B-0FDC-9488-44B62B2747D0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>88900</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>266700</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Chart 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EA78BD48-D418-7D4B-BD62-2081506601B6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1347,7 +4223,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8990D63A-A126-C24A-9B4A-765D86C2F454}">
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.1640625" bestFit="1" customWidth="1"/>
@@ -1355,6 +4231,7 @@
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="10.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -1450,14 +4327,138 @@
         <v>56</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H21" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I21">
+        <f>SUMIF(Expense!$B$2:$B$13,Dashboard!H21,Expense!$D$2:$D$13)</f>
+        <v>355000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H22" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I22">
+        <f>SUMIF(Expense!$B$2:$B$13,Dashboard!H22,Expense!$D$2:$D$13)</f>
+        <v>70000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H23" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I23">
+        <f>SUMIF(Expense!$B$2:$B$13,Dashboard!H23,Expense!$D$2:$D$13)</f>
+        <v>6050000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H24" t="s">
+        <v>13</v>
+      </c>
+      <c r="I24">
+        <f>SUMIF(Expense!$B$2:$B$13,Dashboard!H24,Expense!$D$2:$D$13)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H25" t="s">
+        <v>14</v>
+      </c>
+      <c r="I25">
+        <f>SUMIF(Expense!$B$2:$B$13,Dashboard!H25,Expense!$D$2:$D$13)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H26" t="s">
+        <v>15</v>
+      </c>
+      <c r="I26">
+        <f>SUMIF(Expense!$B$2:$B$13,Dashboard!H26,Expense!$D$2:$D$13)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H27" t="s">
+        <v>16</v>
+      </c>
+      <c r="I27">
+        <f>SUMIF(Expense!$B$2:$B$13,Dashboard!H27,Expense!$D$2:$D$13)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H28" t="s">
+        <v>17</v>
+      </c>
+      <c r="I28">
+        <f>SUMIF(Expense!$B$2:$B$13,Dashboard!H28,Expense!$D$2:$D$13)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H29" t="s">
+        <v>20</v>
+      </c>
+      <c r="I29">
+        <f>SUMIF(Expense!$B$2:$B$13,Dashboard!H29,Expense!$D$2:$D$13)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
         <v>58</v>
+      </c>
+      <c r="H30" t="s">
+        <v>19</v>
+      </c>
+      <c r="I30">
+        <f>SUMIF(Expense!$B$2:$B$13,Dashboard!H30,Expense!$D$2:$D$13)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H31" t="s">
+        <v>21</v>
+      </c>
+      <c r="I31">
+        <f>SUMIF(Expense!$B$2:$B$13,Dashboard!H31,Expense!$D$2:$D$13)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H32" t="s">
+        <v>22</v>
+      </c>
+      <c r="I32">
+        <f>SUMIF(Expense!$B$2:$B$13,Dashboard!H32,Expense!$D$2:$D$13)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H33" t="s">
+        <v>23</v>
+      </c>
+      <c r="I33">
+        <f>SUMIF(Expense!$B$2:$B$13,Dashboard!H33,Expense!$D$2:$D$13)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H34" t="s">
+        <v>24</v>
+      </c>
+      <c r="I34">
+        <f>SUMIF(Expense!$B$2:$B$13,Dashboard!H34,Expense!$D$2:$D$13)</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1470,5 +4471,6 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Day 9: break-even and scenarios
</commit_message>
<xml_diff>
--- a/niasap-data.xlsx
+++ b/niasap-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/metodiuswaruwu/Documents/Project AI/AI-Portofolio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{634F9F22-E164-8847-8D53-9D4E1C57504A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD6A948D-89A6-0640-ADFC-9E21DF10998B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19380" yWindow="720" windowWidth="10000" windowHeight="17160" firstSheet="2" activeTab="5" xr2:uid="{9BF11571-3D57-C340-BE5B-8CD2BEA4A557}"/>
+    <workbookView xWindow="17160" yWindow="720" windowWidth="12220" windowHeight="17160" firstSheet="2" activeTab="6" xr2:uid="{9BF11571-3D57-C340-BE5B-8CD2BEA4A557}"/>
   </bookViews>
   <sheets>
     <sheet name="Sales" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,8 @@
     <sheet name="Category" sheetId="4" r:id="rId4"/>
     <sheet name="Dashboard" sheetId="5" r:id="rId5"/>
     <sheet name="LabaRugi" sheetId="6" r:id="rId6"/>
+    <sheet name="BreakEven" sheetId="7" r:id="rId7"/>
+    <sheet name="Sheet4" sheetId="8" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlchart.v2.0" hidden="1">Sales!$A$2:$A$8</definedName>
@@ -48,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="81">
   <si>
     <t>Tanggal</t>
   </si>
@@ -248,9 +250,6 @@
     <t>Margin Kotor %</t>
   </si>
   <si>
-    <t>Biaya Operasional</t>
-  </si>
-  <si>
     <t>Total Biaya Operasional</t>
   </si>
   <si>
@@ -267,6 +266,33 @@
   </si>
   <si>
     <t>Kertas Nasi</t>
+  </si>
+  <si>
+    <t>Total Biaya Operasional (Fixed)</t>
+  </si>
+  <si>
+    <t>Pendapatan Break-Even (bulanan)</t>
+  </si>
+  <si>
+    <t>Pendapatan Break-Even (Harian)</t>
+  </si>
+  <si>
+    <t>Scenario</t>
+  </si>
+  <si>
+    <t>Monthly Revenue</t>
+  </si>
+  <si>
+    <t>Sepi (Quite)</t>
+  </si>
+  <si>
+    <t>Normal</t>
+  </si>
+  <si>
+    <t>Ramai (Strong)</t>
+  </si>
+  <si>
+    <t>Biaya Operasional (Fix Cost)</t>
   </si>
 </sst>
 </file>
@@ -327,13 +353,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3899,7 +3926,7 @@
         <v>46326</v>
       </c>
       <c r="B7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C7" t="s">
         <v>32</v>
@@ -4018,10 +4045,10 @@
         <v>46327</v>
       </c>
       <c r="B14" t="s">
+        <v>70</v>
+      </c>
+      <c r="C14" t="s">
         <v>71</v>
-      </c>
-      <c r="C14" t="s">
-        <v>72</v>
       </c>
       <c r="D14">
         <v>100000</v>
@@ -4421,7 +4448,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="H24" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I24">
         <f>SUMIF(Expense!$B$2:$B$16,Dashboard!H24,Expense!$D$2:$D$16)</f>
@@ -4676,7 +4703,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
@@ -4773,7 +4800,7 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B28" s="4">
         <f>SUM(B18:B27)</f>
@@ -4786,7 +4813,7 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B30" s="4">
         <f>B14-B28</f>
@@ -4796,7 +4823,7 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B31" s="3">
         <f>B30/B5</f>
@@ -4807,4 +4834,113 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D03D4AA-5D13-F042-9A2F-F90DDDB4C737}">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B1" s="4">
+        <f>LabaRugi!B28</f>
+        <v>4359125</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B2" s="6">
+        <f>LabaRugi!B15</f>
+        <v>0.50264750378214829</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B4" s="4">
+        <f>LabaRugi!B28/LabaRugi!B15</f>
+        <v>8672329.947328819</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5" s="4">
+        <f>B4/30</f>
+        <v>289077.66491096065</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" s="4">
+        <f>B4*0.8</f>
+        <v>6937863.9578630552</v>
+      </c>
+      <c r="C8" s="4">
+        <f>B8*LabaRugi!B15-LabaRugi!B28</f>
+        <v>-871824.99999999953</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9" s="4">
+        <f>B4*1.2</f>
+        <v>10406795.936794583</v>
+      </c>
+      <c r="C9" s="4">
+        <f>B9*LabaRugi!B15-LabaRugi!B28</f>
+        <v>871825</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" s="4">
+        <f>B4*1.6</f>
+        <v>13875727.91572611</v>
+      </c>
+      <c r="C10" s="4">
+        <f>B10*LabaRugi!B15-LabaRugi!B28</f>
+        <v>2615475.0000000009</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3F7A397-A1DC-1641-B1B3-7C11BDC3F561}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>